<commit_message>
Added axes of variation in quadrat IDing conventions
</commit_message>
<xml_diff>
--- a/evaluation/function_inventory.xlsx
+++ b/evaluation/function_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabriela/Dropbox/PERSONAL/LLC/Oikobit LLC/projects/code-and-statistics-forestgeo/fgeo2/evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35D2ADA9-2791-8249-80EC-CFD5BE41BDD1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30713185-D87C-6040-A662-099A4472E63D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3460" yWindow="980" windowWidth="31940" windowHeight="18720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3440" yWindow="980" windowWidth="31940" windowHeight="18720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="functions" sheetId="1" r:id="rId1"/>
@@ -3162,7 +3162,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G372"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -7108,7 +7107,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="232" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>15</v>
       </c>
@@ -7125,7 +7124,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="233" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>18</v>
       </c>
@@ -7142,7 +7141,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="234" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>20</v>
       </c>
@@ -7159,7 +7158,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="235" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>22</v>
       </c>
@@ -7176,7 +7175,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="236" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>24</v>
       </c>
@@ -7193,7 +7192,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="237" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>91</v>
       </c>
@@ -7210,7 +7209,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="238" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>93</v>
       </c>
@@ -7227,7 +7226,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="239" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>132</v>
       </c>
@@ -7244,7 +7243,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="240" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>215</v>
       </c>
@@ -7261,7 +7260,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="241" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>572</v>
       </c>
@@ -7278,7 +7277,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="242" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>560</v>
       </c>
@@ -7295,7 +7294,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="243" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>597</v>
       </c>
@@ -7312,7 +7311,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="244" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>718</v>
       </c>
@@ -7329,7 +7328,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="245" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>720</v>
       </c>
@@ -7346,7 +7345,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="246" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>721</v>
       </c>
@@ -7363,7 +7362,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="247" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>532</v>
       </c>
@@ -7386,7 +7385,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="248" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>535</v>
       </c>
@@ -7409,7 +7408,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="249" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>160</v>
       </c>
@@ -7426,7 +7425,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="250" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>188</v>
       </c>
@@ -7443,7 +7442,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="251" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>237</v>
       </c>
@@ -7460,7 +7459,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="252" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>299</v>
       </c>
@@ -7477,7 +7476,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="253" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>301</v>
       </c>
@@ -7494,7 +7493,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="254" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>319</v>
       </c>
@@ -7511,7 +7510,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="255" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>329</v>
       </c>
@@ -7528,7 +7527,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="256" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>331</v>
       </c>
@@ -7545,7 +7544,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="257" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
         <v>376</v>
       </c>
@@ -7562,7 +7561,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="258" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
         <v>377</v>
       </c>
@@ -7579,7 +7578,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="259" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
         <v>379</v>
       </c>
@@ -7596,7 +7595,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="260" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
         <v>381</v>
       </c>
@@ -7613,7 +7612,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="261" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
         <v>383</v>
       </c>
@@ -7630,7 +7629,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="262" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
         <v>401</v>
       </c>
@@ -7647,7 +7646,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="263" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
         <v>403</v>
       </c>
@@ -7664,7 +7663,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="264" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
         <v>479</v>
       </c>
@@ -7681,7 +7680,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="265" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
         <v>537</v>
       </c>
@@ -7698,7 +7697,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="266" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
         <v>588</v>
       </c>
@@ -7715,7 +7714,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="267" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
         <v>643</v>
       </c>
@@ -7732,7 +7731,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="268" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
         <v>708</v>
       </c>
@@ -7749,7 +7748,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="269" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A269" t="s">
         <v>32</v>
       </c>
@@ -7772,7 +7771,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="270" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A270" t="s">
         <v>114</v>
       </c>
@@ -7795,7 +7794,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="271" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A271" t="s">
         <v>138</v>
       </c>
@@ -7818,7 +7817,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="272" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A272" t="s">
         <v>551</v>
       </c>
@@ -7841,7 +7840,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="273" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
         <v>637</v>
       </c>
@@ -7864,7 +7863,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="274" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A274" t="s">
         <v>179</v>
       </c>
@@ -7881,7 +7880,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="275" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A275" t="s">
         <v>358</v>
       </c>
@@ -7898,7 +7897,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="276" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A276" t="s">
         <v>664</v>
       </c>
@@ -7915,7 +7914,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="277" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A277" t="s">
         <v>666</v>
       </c>
@@ -7932,7 +7931,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="278" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A278" t="s">
         <v>668</v>
       </c>
@@ -7949,7 +7948,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="279" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A279" t="s">
         <v>688</v>
       </c>
@@ -7966,7 +7965,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="280" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A280" t="s">
         <v>0</v>
       </c>
@@ -7983,7 +7982,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="281" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A281" t="s">
         <v>3</v>
       </c>
@@ -8000,7 +7999,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="282" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A282" t="s">
         <v>5</v>
       </c>
@@ -8017,7 +8016,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="283" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A283" t="s">
         <v>7</v>
       </c>
@@ -8034,7 +8033,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="284" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A284" t="s">
         <v>61</v>
       </c>
@@ -8051,7 +8050,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="285" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A285" t="s">
         <v>76</v>
       </c>
@@ -8068,7 +8067,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="286" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A286" t="s">
         <v>567</v>
       </c>
@@ -8085,7 +8084,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="287" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A287" t="s">
         <v>568</v>
       </c>
@@ -8102,7 +8101,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="288" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A288" t="s">
         <v>9</v>
       </c>
@@ -8119,7 +8118,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="289" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A289" t="s">
         <v>63</v>
       </c>
@@ -8136,7 +8135,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="290" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A290" t="s">
         <v>65</v>
       </c>
@@ -8153,7 +8152,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="291" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A291" t="s">
         <v>297</v>
       </c>
@@ -8170,7 +8169,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="292" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A292" t="s">
         <v>311</v>
       </c>
@@ -8187,7 +8186,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="293" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A293" t="s">
         <v>315</v>
       </c>
@@ -8204,7 +8203,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="294" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A294" t="s">
         <v>344</v>
       </c>
@@ -8221,7 +8220,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="295" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A295" t="s">
         <v>389</v>
       </c>
@@ -8238,7 +8237,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="296" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A296" t="s">
         <v>391</v>
       </c>
@@ -8255,7 +8254,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="297" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A297" t="s">
         <v>515</v>
       </c>
@@ -8272,7 +8271,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="298" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A298" t="s">
         <v>574</v>
       </c>
@@ -8289,7 +8288,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="299" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A299" t="s">
         <v>686</v>
       </c>
@@ -8306,7 +8305,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="300" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A300" t="s">
         <v>111</v>
       </c>
@@ -8323,7 +8322,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="301" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A301" t="s">
         <v>405</v>
       </c>
@@ -8340,7 +8339,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="302" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A302" t="s">
         <v>407</v>
       </c>
@@ -8357,7 +8356,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="303" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
         <v>452</v>
       </c>
@@ -8374,7 +8373,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="304" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A304" t="s">
         <v>453</v>
       </c>
@@ -8391,7 +8390,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="305" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A305" t="s">
         <v>95</v>
       </c>
@@ -8408,7 +8407,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="306" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A306" t="s">
         <v>203</v>
       </c>
@@ -8425,7 +8424,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="307" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A307" t="s">
         <v>362</v>
       </c>
@@ -8442,7 +8441,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="308" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A308" t="s">
         <v>364</v>
       </c>
@@ -8459,7 +8458,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="309" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A309" t="s">
         <v>366</v>
       </c>
@@ -8476,7 +8475,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="310" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A310" t="s">
         <v>368</v>
       </c>
@@ -8493,7 +8492,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="311" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A311" t="s">
         <v>372</v>
       </c>
@@ -8510,7 +8509,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="312" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A312" t="s">
         <v>712</v>
       </c>
@@ -8527,7 +8526,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="313" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A313" t="s">
         <v>47</v>
       </c>
@@ -8544,7 +8543,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="314" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A314" t="s">
         <v>67</v>
       </c>
@@ -8561,7 +8560,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="315" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A315" t="s">
         <v>69</v>
       </c>
@@ -8578,7 +8577,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="316" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A316" t="s">
         <v>120</v>
       </c>
@@ -8595,7 +8594,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="317" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A317" t="s">
         <v>122</v>
       </c>
@@ -8612,7 +8611,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="318" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A318" t="s">
         <v>124</v>
       </c>
@@ -8629,7 +8628,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="319" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A319" t="s">
         <v>211</v>
       </c>
@@ -8646,7 +8645,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="320" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A320" t="s">
         <v>213</v>
       </c>
@@ -8663,7 +8662,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="321" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A321" t="s">
         <v>274</v>
       </c>
@@ -8680,7 +8679,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="322" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A322" t="s">
         <v>286</v>
       </c>
@@ -8697,7 +8696,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="323" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A323" t="s">
         <v>370</v>
       </c>
@@ -8714,7 +8713,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="324" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A324" t="s">
         <v>443</v>
       </c>
@@ -8731,7 +8730,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="325" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A325" t="s">
         <v>652</v>
       </c>
@@ -8748,7 +8747,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="326" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A326" t="s">
         <v>654</v>
       </c>
@@ -8765,7 +8764,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="327" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A327" t="s">
         <v>737</v>
       </c>
@@ -8782,7 +8781,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="328" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A328" t="s">
         <v>84</v>
       </c>
@@ -8799,7 +8798,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="329" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A329" t="s">
         <v>87</v>
       </c>
@@ -8816,7 +8815,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="330" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A330" t="s">
         <v>89</v>
       </c>
@@ -8833,7 +8832,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="331" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A331" t="s">
         <v>147</v>
       </c>
@@ -8850,7 +8849,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="332" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A332" t="s">
         <v>346</v>
       </c>
@@ -8867,7 +8866,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="333" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A333" t="s">
         <v>348</v>
       </c>
@@ -8884,7 +8883,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="334" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A334" t="s">
         <v>354</v>
       </c>
@@ -8901,7 +8900,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="335" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A335" t="s">
         <v>356</v>
       </c>
@@ -8918,7 +8917,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="336" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A336" t="s">
         <v>547</v>
       </c>
@@ -8935,7 +8934,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="337" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A337" t="s">
         <v>292</v>
       </c>
@@ -8952,7 +8951,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="338" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A338" t="s">
         <v>522</v>
       </c>
@@ -8969,7 +8968,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="339" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A339" t="s">
         <v>524</v>
       </c>
@@ -8986,7 +8985,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="340" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A340" t="s">
         <v>526</v>
       </c>
@@ -9003,7 +9002,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="341" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A341" t="s">
         <v>528</v>
       </c>
@@ -9020,7 +9019,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="342" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A342" t="s">
         <v>607</v>
       </c>
@@ -9037,7 +9036,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="343" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A343" t="s">
         <v>610</v>
       </c>
@@ -9054,7 +9053,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="344" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A344" t="s">
         <v>239</v>
       </c>
@@ -9071,7 +9070,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="345" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A345" t="s">
         <v>325</v>
       </c>
@@ -9088,7 +9087,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="346" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A346" t="s">
         <v>399</v>
       </c>
@@ -9105,7 +9104,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="347" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A347" t="s">
         <v>660</v>
       </c>
@@ -9122,7 +9121,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="348" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A348" t="s">
         <v>26</v>
       </c>
@@ -9139,7 +9138,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="349" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A349" t="s">
         <v>104</v>
       </c>
@@ -9156,7 +9155,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="350" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A350" t="s">
         <v>106</v>
       </c>
@@ -9173,7 +9172,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="351" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A351" t="s">
         <v>118</v>
       </c>
@@ -9190,7 +9189,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="352" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A352" t="s">
         <v>270</v>
       </c>
@@ -9207,7 +9206,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="353" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A353" t="s">
         <v>590</v>
       </c>
@@ -9224,7 +9223,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="354" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A354" t="s">
         <v>601</v>
       </c>
@@ -9241,7 +9240,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="355" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A355" t="s">
         <v>333</v>
       </c>
@@ -9258,7 +9257,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="356" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A356" t="s">
         <v>603</v>
       </c>
@@ -9275,7 +9274,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="357" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A357" t="s">
         <v>682</v>
       </c>
@@ -9292,7 +9291,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="358" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A358" t="s">
         <v>149</v>
       </c>
@@ -9309,7 +9308,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="359" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A359" t="s">
         <v>209</v>
       </c>
@@ -9326,7 +9325,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="360" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A360" t="s">
         <v>327</v>
       </c>
@@ -9343,7 +9342,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="361" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A361" t="s">
         <v>487</v>
       </c>
@@ -9360,7 +9359,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="362" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A362" t="s">
         <v>489</v>
       </c>
@@ -9377,7 +9376,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="363" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A363" t="s">
         <v>491</v>
       </c>
@@ -9394,7 +9393,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="364" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A364" t="s">
         <v>493</v>
       </c>
@@ -9411,7 +9410,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="365" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A365" t="s">
         <v>553</v>
       </c>
@@ -9428,7 +9427,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="366" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A366" t="s">
         <v>563</v>
       </c>
@@ -9445,7 +9444,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="367" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A367" t="s">
         <v>669</v>
       </c>
@@ -9462,7 +9461,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="368" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A368" t="s">
         <v>142</v>
       </c>
@@ -9479,7 +9478,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="369" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A369" t="s">
         <v>260</v>
       </c>
@@ -9496,7 +9495,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="370" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A370" t="s">
         <v>395</v>
       </c>
@@ -9513,7 +9512,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="371" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A371" t="s">
         <v>397</v>
       </c>
@@ -9530,7 +9529,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="372" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A372" t="s">
         <v>692</v>
       </c>
@@ -9546,11 +9545,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G372" xr:uid="{6BAAEFF7-3956-CB4E-95CA-4544906C3B79}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="01_utilities"/>
-      </filters>
-    </filterColumn>
     <sortState ref="A2:G372">
       <sortCondition ref="B1:B372"/>
     </sortState>

</xml_diff>

<commit_message>
small changes related to dependencies on old quadrat functions
</commit_message>
<xml_diff>
--- a/evaluation/function_inventory.xlsx
+++ b/evaluation/function_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabriela/Dropbox/PERSONAL/LLC/Oikobit LLC/projects/code-and-statistics-forestgeo/fgeo2/evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30713185-D87C-6040-A662-099A4472E63D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AEFF6A2-8DCB-6B4A-B8AD-07BF05C0BCA8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3440" yWindow="980" windowWidth="31940" windowHeight="18720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2040" yWindow="980" windowWidth="33340" windowHeight="18520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="functions" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1883" uniqueCount="766">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1932" uniqueCount="779">
   <si>
     <t>abund.manycensus</t>
   </si>
@@ -2322,6 +2322,45 @@
   </si>
   <si>
     <t>not evaluated</t>
+  </si>
+  <si>
+    <t>NONE</t>
+  </si>
+  <si>
+    <t>Would be covered by more general application of torus translation null models, see https://github.com/gabrielareto/fgeo2/issues/3</t>
+  </si>
+  <si>
+    <t>See quadrats.qmd for examples on how to identiify neighboring quadrats and make community summaries from them</t>
+  </si>
+  <si>
+    <t>quadrats.R</t>
+  </si>
+  <si>
+    <t>Trivial calculation of distances between centroids. See quadrats.qmd for examples on how to calculate distances between quadrats.</t>
+  </si>
+  <si>
+    <t>Trivial -- use expand.grid() in base R</t>
+  </si>
+  <si>
+    <t>All ways of splitting a plot, naming quadrats, transformations local &lt;-&gt; global coordinates, are handled in a more general way with fewer functions. See quadrats.qmd for use cases.</t>
+  </si>
+  <si>
+    <t>Edited so it depends on the new functions to handle quadrats.</t>
+  </si>
+  <si>
+    <t>Removed dependency on deprecated and trivial convert.rowcol()</t>
+  </si>
+  <si>
+    <t>The function is not used by anything else, does not seem relevant</t>
+  </si>
+  <si>
+    <t>Edited to remove dependency on the deprecated gxgy.to.index()</t>
+  </si>
+  <si>
+    <t>See quadrats.qmd for equivalent use cases</t>
+  </si>
+  <si>
+    <t>Minor functionality with obsolete dependencies, both internal and external. Nothing depends on it</t>
   </si>
 </sst>
 </file>
@@ -3996,7 +4035,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>309</v>
       </c>
@@ -4013,7 +4052,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>352</v>
       </c>
@@ -4027,10 +4066,16 @@
         <v>353</v>
       </c>
       <c r="E50" t="s">
-        <v>765</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+        <v>762</v>
+      </c>
+      <c r="F50" t="s">
+        <v>766</v>
+      </c>
+      <c r="G50" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>416</v>
       </c>
@@ -4047,7 +4092,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>431</v>
       </c>
@@ -4064,7 +4109,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>433</v>
       </c>
@@ -4081,7 +4126,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>434</v>
       </c>
@@ -4098,7 +4143,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>435</v>
       </c>
@@ -4115,7 +4160,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>437</v>
       </c>
@@ -4132,7 +4177,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>457</v>
       </c>
@@ -4149,7 +4194,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>461</v>
       </c>
@@ -4166,7 +4211,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>463</v>
       </c>
@@ -4183,7 +4228,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>465</v>
       </c>
@@ -4200,7 +4245,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>467</v>
       </c>
@@ -4217,7 +4262,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>469</v>
       </c>
@@ -4234,7 +4279,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>470</v>
       </c>
@@ -4251,7 +4296,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>472</v>
       </c>
@@ -7310,6 +7355,9 @@
       <c r="E243" t="s">
         <v>765</v>
       </c>
+      <c r="G243" t="s">
+        <v>776</v>
+      </c>
     </row>
     <row r="244" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
@@ -7422,7 +7470,13 @@
         <v>162</v>
       </c>
       <c r="E249" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F249" t="s">
+        <v>769</v>
+      </c>
+      <c r="G249" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="250" spans="1:7" x14ac:dyDescent="0.2">
@@ -7439,7 +7493,13 @@
         <v>189</v>
       </c>
       <c r="E250" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F250" t="s">
+        <v>766</v>
+      </c>
+      <c r="G250" t="s">
+        <v>768</v>
       </c>
     </row>
     <row r="251" spans="1:7" x14ac:dyDescent="0.2">
@@ -7456,7 +7516,13 @@
         <v>238</v>
       </c>
       <c r="E251" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F251" t="s">
+        <v>766</v>
+      </c>
+      <c r="G251" t="s">
+        <v>770</v>
       </c>
     </row>
     <row r="252" spans="1:7" x14ac:dyDescent="0.2">
@@ -7473,7 +7539,13 @@
         <v>300</v>
       </c>
       <c r="E252" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F252" t="s">
+        <v>766</v>
+      </c>
+      <c r="G252" t="s">
+        <v>768</v>
       </c>
     </row>
     <row r="253" spans="1:7" x14ac:dyDescent="0.2">
@@ -7490,7 +7562,13 @@
         <v>302</v>
       </c>
       <c r="E253" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F253" t="s">
+        <v>766</v>
+      </c>
+      <c r="G253" t="s">
+        <v>768</v>
       </c>
     </row>
     <row r="254" spans="1:7" x14ac:dyDescent="0.2">
@@ -7507,7 +7585,13 @@
         <v>320</v>
       </c>
       <c r="E254" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F254" t="s">
+        <v>766</v>
+      </c>
+      <c r="G254" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="255" spans="1:7" x14ac:dyDescent="0.2">
@@ -7524,7 +7608,13 @@
         <v>330</v>
       </c>
       <c r="E255" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F255" t="s">
+        <v>769</v>
+      </c>
+      <c r="G255" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="256" spans="1:7" x14ac:dyDescent="0.2">
@@ -7541,7 +7631,13 @@
         <v>332</v>
       </c>
       <c r="E256" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F256" t="s">
+        <v>769</v>
+      </c>
+      <c r="G256" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="257" spans="1:7" x14ac:dyDescent="0.2">
@@ -7558,7 +7654,13 @@
         <v>70</v>
       </c>
       <c r="E257" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F257" t="s">
+        <v>769</v>
+      </c>
+      <c r="G257" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.2">
@@ -7575,7 +7677,13 @@
         <v>378</v>
       </c>
       <c r="E258" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F258" t="s">
+        <v>769</v>
+      </c>
+      <c r="G258" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="259" spans="1:7" x14ac:dyDescent="0.2">
@@ -7592,7 +7700,13 @@
         <v>380</v>
       </c>
       <c r="E259" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F259" t="s">
+        <v>769</v>
+      </c>
+      <c r="G259" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="260" spans="1:7" x14ac:dyDescent="0.2">
@@ -7609,7 +7723,13 @@
         <v>382</v>
       </c>
       <c r="E260" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F260" t="s">
+        <v>769</v>
+      </c>
+      <c r="G260" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="261" spans="1:7" x14ac:dyDescent="0.2">
@@ -7626,7 +7746,13 @@
         <v>384</v>
       </c>
       <c r="E261" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F261" t="s">
+        <v>769</v>
+      </c>
+      <c r="G261" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="262" spans="1:7" x14ac:dyDescent="0.2">
@@ -7643,7 +7769,13 @@
         <v>402</v>
       </c>
       <c r="E262" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F262" t="s">
+        <v>769</v>
+      </c>
+      <c r="G262" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="263" spans="1:7" x14ac:dyDescent="0.2">
@@ -7660,7 +7792,13 @@
         <v>404</v>
       </c>
       <c r="E263" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F263" t="s">
+        <v>769</v>
+      </c>
+      <c r="G263" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="264" spans="1:7" x14ac:dyDescent="0.2">
@@ -7677,7 +7815,13 @@
         <v>480</v>
       </c>
       <c r="E264" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F264" t="s">
+        <v>769</v>
+      </c>
+      <c r="G264" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.2">
@@ -7694,7 +7838,13 @@
         <v>538</v>
       </c>
       <c r="E265" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F265" t="s">
+        <v>766</v>
+      </c>
+      <c r="G265" t="s">
+        <v>768</v>
       </c>
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.2">
@@ -7711,7 +7861,13 @@
         <v>589</v>
       </c>
       <c r="E266" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F266" t="s">
+        <v>769</v>
+      </c>
+      <c r="G266" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="267" spans="1:7" x14ac:dyDescent="0.2">
@@ -7728,7 +7884,13 @@
         <v>208</v>
       </c>
       <c r="E267" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F267" t="s">
+        <v>769</v>
+      </c>
+      <c r="G267" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="268" spans="1:7" x14ac:dyDescent="0.2">
@@ -7745,7 +7907,13 @@
         <v>709</v>
       </c>
       <c r="E268" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F268" t="s">
+        <v>766</v>
+      </c>
+      <c r="G268" t="s">
+        <v>767</v>
       </c>
     </row>
     <row r="269" spans="1:7" x14ac:dyDescent="0.2">
@@ -7928,7 +8096,13 @@
         <v>667</v>
       </c>
       <c r="E277" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F277" t="s">
+        <v>766</v>
+      </c>
+      <c r="G277" t="s">
+        <v>775</v>
       </c>
     </row>
     <row r="278" spans="1:7" x14ac:dyDescent="0.2">
@@ -8030,7 +8204,13 @@
         <v>8</v>
       </c>
       <c r="E283" t="s">
-        <v>765</v>
+        <v>762</v>
+      </c>
+      <c r="F283" t="s">
+        <v>766</v>
+      </c>
+      <c r="G283" t="s">
+        <v>777</v>
       </c>
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.2">
@@ -8934,7 +9114,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A337" t="s">
         <v>292</v>
       </c>
@@ -8951,7 +9131,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A338" t="s">
         <v>522</v>
       </c>
@@ -8968,7 +9148,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A339" t="s">
         <v>524</v>
       </c>
@@ -8985,7 +9165,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A340" t="s">
         <v>526</v>
       </c>
@@ -9002,7 +9182,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A341" t="s">
         <v>528</v>
       </c>
@@ -9019,7 +9199,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A342" t="s">
         <v>607</v>
       </c>
@@ -9036,7 +9216,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A343" t="s">
         <v>610</v>
       </c>
@@ -9053,7 +9233,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A344" t="s">
         <v>239</v>
       </c>
@@ -9070,7 +9250,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A345" t="s">
         <v>325</v>
       </c>
@@ -9086,8 +9266,11 @@
       <c r="E345" t="s">
         <v>765</v>
       </c>
-    </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G345" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="346" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A346" t="s">
         <v>399</v>
       </c>
@@ -9104,7 +9287,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A347" t="s">
         <v>660</v>
       </c>
@@ -9121,7 +9304,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A348" t="s">
         <v>26</v>
       </c>
@@ -9137,8 +9320,11 @@
       <c r="E348" t="s">
         <v>765</v>
       </c>
-    </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G348" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="349" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A349" t="s">
         <v>104</v>
       </c>
@@ -9155,7 +9341,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A350" t="s">
         <v>106</v>
       </c>
@@ -9172,7 +9358,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A351" t="s">
         <v>118</v>
       </c>
@@ -9189,7 +9375,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A352" t="s">
         <v>270</v>
       </c>

</xml_diff>